<commit_message>
Modified Task 7 to have better Risk of Overflow analysis. Updataed data collected
</commit_message>
<xml_diff>
--- a/Practical3/STM32F0_Task7_Data.xlsx
+++ b/Practical3/STM32F0_Task7_Data.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://uctcloud-my.sharepoint.com/personal/ngrmar007_myuct_ac_za/Documents/Third Year/EEE3096s-repository/EEE3096S-Group-39/Practical3/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="5" documentId="8_{A96F95B7-3D4F-43BC-8035-7A878770923F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{6E0DCEF8-016D-40FA-87BD-B854EE1B636A}"/>
+  <xr:revisionPtr revIDLastSave="17" documentId="8_{A96F95B7-3D4F-43BC-8035-7A878770923F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{9BA44081-F0D4-459D-8368-7214E7B8AA18}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{DCD1EBFB-3F9F-4111-B99B-084E4A1C7696}"/>
+    <workbookView xWindow="11424" yWindow="0" windowWidth="11712" windowHeight="12336" xr2:uid="{DCD1EBFB-3F9F-4111-B99B-084E4A1C7696}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -115,6 +115,10 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -437,357 +441,357 @@
   <dimension ref="A1:G16"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="17.33203125" style="2" customWidth="1"/>
-    <col min="2" max="2" width="16.109375" style="2" customWidth="1"/>
-    <col min="3" max="3" width="32.33203125" style="2" customWidth="1"/>
-    <col min="4" max="4" width="35.21875" style="2" customWidth="1"/>
-    <col min="5" max="5" width="21.21875" style="2" customWidth="1"/>
-    <col min="6" max="6" width="30.109375" style="2" customWidth="1"/>
-    <col min="7" max="7" width="27.6640625" style="2" customWidth="1"/>
+    <col min="1" max="1" width="17.33203125" style="1" customWidth="1"/>
+    <col min="2" max="2" width="16.109375" style="1" customWidth="1"/>
+    <col min="3" max="3" width="32.33203125" style="1" customWidth="1"/>
+    <col min="4" max="4" width="35.21875" style="1" customWidth="1"/>
+    <col min="5" max="5" width="21.21875" style="1" customWidth="1"/>
+    <col min="6" max="6" width="30.109375" style="1" customWidth="1"/>
+    <col min="7" max="7" width="27.6640625" style="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A1" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="2" t="s">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="2" t="s">
+      <c r="C1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="D1" s="2" t="s">
+      <c r="D1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="E1" s="2" t="s">
+      <c r="E1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="2" t="s">
+      <c r="F1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="G1" s="2" t="s">
+      <c r="G1" s="1" t="s">
         <v>2</v>
       </c>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A2" s="1">
+      <c r="A2" s="2">
         <v>1000</v>
       </c>
-      <c r="B2" s="2">
+      <c r="B2" s="1">
         <v>128</v>
       </c>
-      <c r="C2" s="2">
+      <c r="C2" s="1">
         <v>20405</v>
       </c>
-      <c r="D2" s="2">
+      <c r="D2" s="1">
         <v>31548</v>
       </c>
-      <c r="E2" s="2">
+      <c r="E2" s="1">
         <v>430441</v>
       </c>
-      <c r="F2" s="2">
-        <v>0</v>
-      </c>
-      <c r="G2" s="2">
+      <c r="F2" s="1">
+        <v>0</v>
+      </c>
+      <c r="G2" s="1">
         <v>0</v>
       </c>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A3" s="1"/>
-      <c r="B3" s="2">
+      <c r="A3" s="2"/>
+      <c r="B3" s="1">
         <v>160</v>
       </c>
-      <c r="C3" s="2">
+      <c r="C3" s="1">
         <v>31891</v>
       </c>
-      <c r="D3" s="2">
+      <c r="D3" s="1">
         <v>49327</v>
       </c>
-      <c r="E3" s="2">
+      <c r="E3" s="1">
         <v>672420</v>
       </c>
-      <c r="F3" s="2">
-        <v>0</v>
-      </c>
-      <c r="G3" s="2">
+      <c r="F3" s="1">
+        <v>0</v>
+      </c>
+      <c r="G3" s="1">
         <v>0</v>
       </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A4" s="1"/>
-      <c r="B4" s="2">
+      <c r="A4" s="2"/>
+      <c r="B4" s="1">
         <v>192</v>
       </c>
-      <c r="C4" s="2">
+      <c r="C4" s="1">
         <v>45923</v>
       </c>
-      <c r="D4" s="2">
+      <c r="D4" s="1">
         <v>71014</v>
       </c>
-      <c r="E4" s="2">
+      <c r="E4" s="1">
         <v>967841</v>
       </c>
-      <c r="F4" s="2">
-        <v>0</v>
-      </c>
-      <c r="G4" s="2">
+      <c r="F4" s="1">
+        <v>0</v>
+      </c>
+      <c r="G4" s="1">
         <v>0</v>
       </c>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A5" s="1"/>
-      <c r="B5" s="2">
+      <c r="A5" s="2"/>
+      <c r="B5" s="1">
         <v>224</v>
       </c>
-      <c r="C5" s="2">
+      <c r="C5" s="1">
         <v>62570</v>
       </c>
-      <c r="D5" s="2">
+      <c r="D5" s="1">
         <v>96713</v>
       </c>
-      <c r="E5" s="2">
+      <c r="E5" s="1">
         <v>1318918</v>
       </c>
-      <c r="F5" s="2">
-        <v>0</v>
-      </c>
-      <c r="G5" s="2">
+      <c r="F5" s="1">
+        <v>0</v>
+      </c>
+      <c r="G5" s="1">
         <v>0</v>
       </c>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A6" s="1"/>
-      <c r="B6" s="2">
+      <c r="A6" s="2"/>
+      <c r="B6" s="1">
         <v>256</v>
       </c>
-      <c r="C6" s="2">
+      <c r="C6" s="1">
         <v>81713</v>
       </c>
-      <c r="D6" s="2">
+      <c r="D6" s="1">
         <v>126335</v>
       </c>
-      <c r="E6" s="2">
+      <c r="E6" s="1">
         <v>1721196</v>
       </c>
-      <c r="F6" s="2">
-        <v>0</v>
-      </c>
-      <c r="G6" s="2">
+      <c r="F6" s="1">
+        <v>0</v>
+      </c>
+      <c r="G6" s="1">
         <v>0</v>
       </c>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A7" s="1">
+      <c r="A7" s="2">
         <v>10000</v>
       </c>
-      <c r="B7" s="2">
+      <c r="B7" s="1">
         <v>128</v>
       </c>
-      <c r="C7" s="2">
+      <c r="C7" s="1">
         <v>22641</v>
       </c>
-      <c r="D7" s="2">
+      <c r="D7" s="1">
         <v>33427</v>
       </c>
-      <c r="E7" s="2">
+      <c r="E7" s="1">
         <v>429902</v>
       </c>
-      <c r="F7" s="2">
-        <v>0</v>
-      </c>
-      <c r="G7" s="2">
+      <c r="F7" s="1">
+        <v>0</v>
+      </c>
+      <c r="G7" s="1">
         <v>0</v>
       </c>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A8" s="1"/>
-      <c r="B8" s="2">
+      <c r="A8" s="2"/>
+      <c r="B8" s="1">
         <v>160</v>
       </c>
-      <c r="C8" s="2">
+      <c r="C8" s="1">
         <v>35352</v>
       </c>
-      <c r="D8" s="2">
+      <c r="D8" s="1">
         <v>52180</v>
       </c>
-      <c r="E8" s="2">
+      <c r="E8" s="1">
         <v>670792</v>
       </c>
-      <c r="F8" s="2">
-        <v>0</v>
-      </c>
-      <c r="G8" s="2">
+      <c r="F8" s="1">
+        <v>0</v>
+      </c>
+      <c r="G8" s="1">
         <v>0</v>
       </c>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A9" s="1"/>
-      <c r="B9" s="2">
+      <c r="A9" s="2"/>
+      <c r="B9" s="1">
         <v>192</v>
       </c>
-      <c r="C9" s="2">
+      <c r="C9" s="1">
         <v>50943</v>
       </c>
-      <c r="D9" s="2">
+      <c r="D9" s="1">
         <v>75194</v>
       </c>
-      <c r="E9" s="2">
+      <c r="E9" s="1">
         <v>966180</v>
       </c>
-      <c r="F9" s="2">
-        <v>0</v>
-      </c>
-      <c r="G9" s="2">
+      <c r="F9" s="1">
+        <v>0</v>
+      </c>
+      <c r="G9" s="1">
         <v>0</v>
       </c>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A10" s="1"/>
-      <c r="B10" s="2">
+      <c r="A10" s="2"/>
+      <c r="B10" s="1">
         <v>224</v>
       </c>
-      <c r="C10" s="2">
+      <c r="C10" s="1">
         <v>69350</v>
       </c>
-      <c r="D10" s="2">
+      <c r="D10" s="1">
         <v>102338</v>
       </c>
-      <c r="E10" s="2">
+      <c r="E10" s="1">
         <v>1315182</v>
       </c>
-      <c r="F10" s="2">
-        <v>0</v>
-      </c>
-      <c r="G10" s="2">
+      <c r="F10" s="1">
+        <v>0</v>
+      </c>
+      <c r="G10" s="1">
         <v>0</v>
       </c>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A11" s="1"/>
-      <c r="B11" s="2">
+      <c r="A11" s="2"/>
+      <c r="B11" s="1">
         <v>256</v>
       </c>
-      <c r="C11" s="2">
+      <c r="C11" s="1">
         <v>90596</v>
       </c>
-      <c r="D11" s="2">
+      <c r="D11" s="1">
         <v>133692</v>
       </c>
-      <c r="E11" s="2">
+      <c r="E11" s="1">
         <v>1716795</v>
       </c>
-      <c r="F11" s="2">
-        <v>0</v>
-      </c>
-      <c r="G11" s="2">
+      <c r="F11" s="1">
+        <v>0</v>
+      </c>
+      <c r="G11" s="1">
         <v>0</v>
       </c>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A12" s="1">
+      <c r="A12" s="2">
         <v>1000000</v>
       </c>
-      <c r="B12" s="2">
+      <c r="B12" s="1">
         <v>128</v>
       </c>
-      <c r="C12" s="2">
+      <c r="C12" s="1">
         <v>24050</v>
       </c>
-      <c r="D12" s="2">
+      <c r="D12" s="1">
         <v>34012</v>
       </c>
-      <c r="E12" s="2">
+      <c r="E12" s="1">
         <v>429346</v>
       </c>
-      <c r="F12" s="2">
-        <v>0</v>
-      </c>
-      <c r="G12" s="2">
-        <v>0</v>
+      <c r="F12" s="1">
+        <v>371924</v>
+      </c>
+      <c r="G12" s="1">
+        <v>387106</v>
       </c>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A13" s="1"/>
-      <c r="B13" s="2">
+      <c r="A13" s="2"/>
+      <c r="B13" s="1">
         <v>160</v>
       </c>
-      <c r="C13" s="2">
+      <c r="C13" s="1">
         <v>37569</v>
       </c>
-      <c r="D13" s="2">
+      <c r="D13" s="1">
         <v>53114</v>
       </c>
-      <c r="E13" s="2">
+      <c r="E13" s="1">
         <v>669809</v>
       </c>
-      <c r="F13" s="2">
-        <v>0</v>
-      </c>
-      <c r="G13" s="2">
-        <v>0</v>
+      <c r="F13" s="1">
+        <v>580982</v>
+      </c>
+      <c r="G13" s="1">
+        <v>605480</v>
       </c>
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A14" s="1"/>
-      <c r="B14" s="2">
+      <c r="A14" s="2"/>
+      <c r="B14" s="1">
         <v>192</v>
       </c>
-      <c r="C14" s="2">
+      <c r="C14" s="1">
         <v>54218</v>
       </c>
-      <c r="D14" s="2">
+      <c r="D14" s="1">
         <v>76648</v>
       </c>
-      <c r="E14" s="2">
+      <c r="E14" s="1">
         <v>966227</v>
       </c>
-      <c r="F14" s="2">
-        <v>0</v>
-      </c>
-      <c r="G14" s="2">
-        <v>0</v>
+      <c r="F14" s="1">
+        <v>838013</v>
+      </c>
+      <c r="G14" s="1">
+        <v>872776</v>
       </c>
     </row>
     <row r="15" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A15" s="1"/>
-      <c r="B15" s="2">
+      <c r="A15" s="2"/>
+      <c r="B15" s="1">
         <v>224</v>
       </c>
-      <c r="C15" s="2">
+      <c r="C15" s="1">
         <v>73822</v>
       </c>
-      <c r="D15" s="2">
+      <c r="D15" s="1">
         <v>104335</v>
       </c>
-      <c r="E15" s="2">
+      <c r="E15" s="1">
         <v>1315085</v>
       </c>
-      <c r="F15" s="2">
-        <v>0</v>
-      </c>
-      <c r="G15" s="2">
-        <v>0</v>
+      <c r="F15" s="1">
+        <v>1140780</v>
+      </c>
+      <c r="G15" s="1">
+        <v>1188052</v>
       </c>
     </row>
     <row r="16" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A16" s="1"/>
-      <c r="B16" s="2">
+      <c r="A16" s="2"/>
+      <c r="B16" s="1">
         <v>256</v>
       </c>
-      <c r="C16" s="2">
+      <c r="C16" s="1">
         <v>96408</v>
       </c>
-      <c r="D16" s="2">
+      <c r="D16" s="1">
         <v>136247</v>
       </c>
-      <c r="E16" s="2">
+      <c r="E16" s="1">
         <v>1715815</v>
       </c>
-      <c r="F16" s="2">
-        <v>0</v>
-      </c>
-      <c r="G16" s="2">
-        <v>0</v>
+      <c r="F16" s="1">
+        <v>1487361</v>
+      </c>
+      <c r="G16" s="1">
+        <v>1551386</v>
       </c>
     </row>
   </sheetData>

</xml_diff>